<commit_message>
test clean & standardise text
</commit_message>
<xml_diff>
--- a/Power BI Data Analyst/Dataset/Contoso Bikes.xlsx
+++ b/Power BI Data Analyst/Dataset/Contoso Bikes.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C93C5F5B-849D-4556-8C11-2CAE0C57DD43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFD742DE-3C81-4936-8246-4A63165D160C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{622B0F4C-E256-446E-B5AC-66D6225C39AF}"/>
   </bookViews>
@@ -1303,35 +1303,13 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="H7:H16" formula="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="ff7972f0-e6b1-4e81-bd6d-6d5a7ea56092">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <MediaLengthInSeconds xmlns="520977d3-e5b6-4195-9522-2071cc7a7d60" xsi:nil="true"/>
-    <_activity xmlns="520977d3-e5b6-4195-9522-2071cc7a7d60" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006D9D3B1A3CBCA94C9C619CD08E0E4046" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9318375d1ce6441558b5f48286c88a85">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="520977d3-e5b6-4195-9522-2071cc7a7d60" xmlns:ns4="ff7972f0-e6b1-4e81-bd6d-6d5a7ea56092" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4e16bed0848fef8ca41883df276aa630" ns3:_="" ns4:_="">
     <xsd:import namespace="520977d3-e5b6-4195-9522-2071cc7a7d60"/>
@@ -1578,32 +1556,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E771D00-F70B-4A71-A745-CFD4425C64F9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="ff7972f0-e6b1-4e81-bd6d-6d5a7ea56092"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="520977d3-e5b6-4195-9522-2071cc7a7d60"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75AEEDF9-0B70-424C-8DA2-B4649D7D6C19}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="ff7972f0-e6b1-4e81-bd6d-6d5a7ea56092">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <MediaLengthInSeconds xmlns="520977d3-e5b6-4195-9522-2071cc7a7d60" xsi:nil="true"/>
+    <_activity xmlns="520977d3-e5b6-4195-9522-2071cc7a7d60" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81B66C32-C8B2-44B2-9B49-E4FBF0E25D3C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1620,4 +1598,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75AEEDF9-0B70-424C-8DA2-B4649D7D6C19}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E771D00-F70B-4A71-A745-CFD4425C64F9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="ff7972f0-e6b1-4e81-bd6d-6d5a7ea56092"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="520977d3-e5b6-4195-9522-2071cc7a7d60"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>